<commit_message>
Caderneta de Poupança e Selic implementadas
Agora a regra da Caderneta de Poupança está funcionando e a Ec 113/2021 já está funcionando, com as colunas devidamente ajustadas. regras.htlm foi ajustado a exibição dos parâmetros. Próxima etapa: ajustar o período de correção.
</commit_message>
<xml_diff>
--- a/arquivos/indices.xlsx
+++ b/arquivos/indices.xlsx
@@ -47,7 +47,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="yyyy\-mm"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -118,10 +118,10 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -13007,7 +13007,7 @@
         <v>40026</v>
       </c>
       <c r="C1145" s="4">
-        <v>1.07</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="1146" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>